<commit_message>
feat: update student Excel template to improve compatibility and data handling
</commit_message>
<xml_diff>
--- a/public/templates/students_template.xlsx
+++ b/public/templates/students_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barrilitodev/Documents/Projects/Rutes/RutEs-Admin/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barrilitodev/Documents/Projects/Rutes/RutEs-Admin/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{693C497B-86C0-D343-80BA-853A665B6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A7161DCA-3155-534F-8A99-B04EBEBEC3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{C0037EC9-82D7-9341-9D99-240AE8B72804}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="29" uniqueCount="29">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="30" uniqueCount="30">
   <si>
     <t>nombre_estudiante</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>existe_madre</t>
+  </si>
+  <si>
+    <t>complete</t>
   </si>
 </sst>
 </file>
@@ -972,7 +975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{438F966A-1D40-CB45-8498-802A5BCD86E5}">
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.2">
@@ -1064,10 +1067,18 @@
         <v>28</v>
       </c>
     </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2 AC2" xr:uid="{C853F37F-465B-9E4D-BF46-11280036C079}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB2:AC2" xr:uid="{C853F37F-465B-9E4D-BF46-11280036C079}">
       <formula1>"Si, No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{9F974F44-E1EF-8C40-ABF8-3CCE8D842DDD}">
+      <formula1>"complete"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>